<commit_message>
Added 4 Test Cases to Excel Sheet
</commit_message>
<xml_diff>
--- a/Team-5_Test-Cases(1).xlsx
+++ b/Team-5_Test-Cases(1).xlsx
@@ -13,10 +13,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={5e04ab7e-e6cb-4a4e-8ec2-5ab0399ec0f2}</author>
+    <author>tc={dac5ceab-4fcd-43b1-aa9a-912570d825cc}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{5e04ab7e-e6cb-4a4e-8ec2-5ab0399ec0f2}" ref="A3">
+    <comment authorId="0" xr:uid="{dac5ceab-4fcd-43b1-aa9a-912570d825cc}" ref="A3">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="92">
   <si>
     <t>Test Cases</t>
   </si>
@@ -185,6 +185,171 @@
   </si>
   <si>
     <t>System rate-limits excessive requests and/or prompts a human verification challenge. If verification is failed, checkout remains blocked. After passing verification (or waiting out rate limit), legitimate checkout can proceed. Security event is logged for admin review.</t>
+  </si>
+  <si>
+    <t>AdminAccessDenial_1</t>
+  </si>
+  <si>
+    <t>Verify that a non-admin user cannot access the admin panel and that the event is correctly logged.</t>
+  </si>
+  <si>
+    <t>Logging is set up and works, test user being a registered user and non registered user exists,</t>
+  </si>
+  <si>
+    <t>1. Log in as a standard registered user.
+2. Directly navigate to the admin panel URL.
+3. Observe the response and page displayed.
+5. Check the security log via admin account for the unauthorized access attempt entry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access is denied with a clear error message and the user is not shown any admin UI or ANY data. An unauthorized access attempt entry is recorded in the security log with timestamp and user identifier </t>
+  </si>
+  <si>
+    <t>Access denied message</t>
+  </si>
+  <si>
+    <t>Pentester</t>
+  </si>
+  <si>
+    <t>PaymentFailure_1</t>
+  </si>
+  <si>
+    <t>Order_Payment_Module</t>
+  </si>
+  <si>
+    <t>Verify that a failed payment does not finalize the order, releases the seat hold, and logs the failure event.</t>
+  </si>
+  <si>
+    <t>Valid showtime exists within purchase window, user is on seat selection page. A open seat is available.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Simulate going to checkout
+2. Observe the order status after declining midway through purchase (like exiting the page before it finishes)
+3. Check the seat status after and that it is available
+4. Check the logs for the payment failure event
+5. Confrim that no confirmation number was issued
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The order remains unconfirmed, the seat is freely available, payment failure logged with the timestamp and ID, </t>
+  </si>
+  <si>
+    <t>Seat is available, and no confirmation number</t>
+  </si>
+  <si>
+    <t>DiscountPricing_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User </t>
+  </si>
+  <si>
+    <t>SeatHoldTimer_1</t>
+  </si>
+  <si>
+    <t>RefundRequest_1</t>
+  </si>
+  <si>
+    <t>Order_Refund_Module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify that a user can successfully request a refund for an order that has already been completed, only within the allowed time for a refund. </t>
+  </si>
+  <si>
+    <t>Valid Order Purchase , Within Order Refund Timeframe, Order Refund Page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Login as Registed User 
+2. Go to order history and click on eligible order  
+3. Request Refund 
+4. Confirm Refund
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The order is refunded. Order changes from being ordered to being refunded, then any items in the order are released and put back into the inventory </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order is Refunded </t>
+  </si>
+  <si>
+    <t>Tester</t>
+  </si>
+  <si>
+    <t>GuestCheckout_1</t>
+  </si>
+  <si>
+    <t>Checkout_Module</t>
+  </si>
+  <si>
+    <t>Verify that a Guest User is able to complete a ticket purchase without needing an account</t>
+  </si>
+  <si>
+    <t>Valid Showtime, Avaliable Seats, Valid Payment Method, Checkout Page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the desired showtime
+2. Confirm seat selection 
+3. Procceed to Checkout 
+4. Checkout as guest 
+5. Confirm details 
+6. Complete Payment </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The order is able to be completed by the guest user without needing to login, User recieves confirmation via Email / SMS 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guest is able to Complete Purchase </t>
+  </si>
+  <si>
+    <t>DiscountCode
+Validation_1</t>
+  </si>
+  <si>
+    <t>Pricing_Module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify if a discount code is expired or invalid, showing appropriate errors for each one. </t>
+  </si>
+  <si>
+    <t>Expired Discount Code, Invalid Discount Code, Checkout Page</t>
+  </si>
+  <si>
+    <t>1. Navigate to checkout 
+2. Enter in expired discount code 
+3. Observe the error popup for expired code
+4. Clear the discount code field and enter invalid discount code 
+5. Observe the error popup for the invalid code entered</t>
+  </si>
+  <si>
+    <t>Neither of the code are accepted when entered in the discount code field. Error message popup saying code is expired or that the code is invalid. The total amount on the order is unaffected.</t>
+  </si>
+  <si>
+    <t>Invalid &amp; Expired Discount Codes are not accepted</t>
+  </si>
+  <si>
+    <t>Email
+Confirmation_1</t>
+  </si>
+  <si>
+    <t>Notification_Module</t>
+  </si>
+  <si>
+    <t>Verify that the Email Confirmation are working as intended right affter the completion of a purchase</t>
+  </si>
+  <si>
+    <t>Valid Email, Purchase just completed, Confirmation Page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to checkout and complete a purchase
+2. Check inbox of designated Email 
+3. Open confirmation Email 
+4. Check that the details in the confirmation Email are the same as the details on the confirmation page </t>
+  </si>
+  <si>
+    <t>Confirmation Email is received within a short time window after the completion of purcahse. Email is showing the correct details(showtime, seat , price, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmation Email recieved </t>
   </si>
 </sst>
 </file>
@@ -340,7 +505,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Victor Lopez" id="{bc6e0f19-7526-4fa8-ae42-d90b77423a9e}" providerId="google-sheets"/>
+  <x18tc:person displayName="Victor Lopez" id="{fb3c67f4-c2b9-4e5f-8dae-10585fa6b1c3}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -540,7 +705,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A3" dT="2026-03-18T03:00:40.00" personId="{bc6e0f19-7526-4fa8-ae42-d90b77423a9e}" id="{5e04ab7e-e6cb-4a4e-8ec2-5ab0399ec0f2}" done="0">
+  <x18tc:threadedComment ref="A3" dT="2026-03-18T03:00:40.00" personId="{fb3c67f4-c2b9-4e5f-8dae-10585fa6b1c3}" id="{dac5ceab-4fcd-43b1-aa9a-912570d825cc}" done="0">
     <x18tc:text xml:space="preserve">Pascal case, underscores for spaces.
 P0 for security testing or anything that is website breaking
 P1 for functionality 
@@ -754,45 +919,87 @@
       <c r="J7" s="5"/>
     </row>
     <row r="8" ht="90.0" customHeight="1">
-      <c r="A8" s="5"/>
+      <c r="A8" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
+      <c r="C8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>51</v>
+      </c>
       <c r="I8" s="8"/>
-      <c r="J8" s="5"/>
+      <c r="J8" s="9" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="9" ht="90.0" customHeight="1">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
+      <c r="A9" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>59</v>
+      </c>
       <c r="I9" s="8"/>
       <c r="J9" s="5"/>
     </row>
     <row r="10" ht="90.0" customHeight="1">
-      <c r="A10" s="5"/>
+      <c r="A10" s="9" t="s">
+        <v>60</v>
+      </c>
       <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
+      <c r="C10" s="9" t="s">
+        <v>23</v>
+      </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="7"/>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
       <c r="I10" s="8"/>
-      <c r="J10" s="5"/>
+      <c r="J10" s="9" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="11" ht="90.0" customHeight="1">
-      <c r="A11" s="5"/>
+      <c r="A11" s="9" t="s">
+        <v>62</v>
+      </c>
       <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
+      <c r="C11" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="7"/>
@@ -802,52 +1009,124 @@
       <c r="J11" s="5"/>
     </row>
     <row r="12" ht="90.0" customHeight="1">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
+      <c r="A12" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>69</v>
+      </c>
       <c r="I12" s="8"/>
-      <c r="J12" s="5"/>
+      <c r="J12" s="9" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="13" ht="90.0" customHeight="1">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
+      <c r="A13" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="I13" s="8"/>
-      <c r="J13" s="5"/>
+      <c r="J13" s="9" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="14" ht="90.0" customHeight="1">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
+      <c r="A14" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>84</v>
+      </c>
       <c r="I14" s="8"/>
-      <c r="J14" s="5"/>
+      <c r="J14" s="9" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="15" ht="90.0" customHeight="1">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
+      <c r="A15" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>91</v>
+      </c>
       <c r="I15" s="8"/>
-      <c r="J15" s="5"/>
+      <c r="J15" s="9" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="16" ht="90.0" customHeight="1">
       <c r="A16" s="5"/>

</xml_diff>

<commit_message>
Added 4 more test cases
</commit_message>
<xml_diff>
--- a/Team-5_Test-Cases(1).xlsx
+++ b/Team-5_Test-Cases(1).xlsx
@@ -13,10 +13,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={dac5ceab-4fcd-43b1-aa9a-912570d825cc}</author>
+    <author>tc={163cf64a-9a5e-4384-8ab6-10911567c6be}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{dac5ceab-4fcd-43b1-aa9a-912570d825cc}" ref="A3">
+    <comment authorId="0" xr:uid="{163cf64a-9a5e-4384-8ab6-10911567c6be}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="104">
   <si>
     <t>Test Cases</t>
   </si>
@@ -68,38 +68,6 @@
   </si>
   <si>
     <t>Test Executed By</t>
-  </si>
-  <si>
-    <t>GoogleSearch_1</t>
-  </si>
-  <si>
-    <t>Search_Bar_Module</t>
-  </si>
-  <si>
-    <t>P0</t>
-  </si>
-  <si>
-    <t>Verify that when a user writes a search term and presses enter, search results should be displayed</t>
-  </si>
-  <si>
-    <t>Browser is launched</t>
-  </si>
-  <si>
-    <t>1. Write the url - http://google.com in the browser's URL bar and press enter.
-2. Once google.com is launched, write the search term - "Apple" in the google search bar.
-3. Press enter.</t>
-  </si>
-  <si>
-    <t>Search results related to 'apple' should be displayed</t>
-  </si>
-  <si>
-    <t>Search results with 'apple' keyword are displayed</t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>CI/CD Pipeline</t>
   </si>
   <si>
     <t>MaxTicketsFunction_1</t>
@@ -126,6 +94,15 @@
     <t>System prevents checkout and displays a clear message indicating the 20-ticket maxmimum per transaction, no seats are sold, and any temporary holds expire normally.</t>
   </si>
   <si>
+    <t>Attempting to purchase 21 tickets was blocked at checkout. System displayed "Maximum 20 Tickets per Transaction." No seats were sold and the transaction did not proceed.</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>CI/CD Pipeline (Functional Test)</t>
+  </si>
+  <si>
     <t>PurchaseWindowFunction_2</t>
   </si>
   <si>
@@ -141,6 +118,12 @@
   </si>
   <si>
     <t>For B: checkout blocked with message “Tickets available 2 weeks prior”. For A: checkout allowed. For C: checkout blocked with message indicating sales close 10 minutes after start.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Showtime 30 days away: Checkout blocked with message indicating tickets available 14 days prior. Showtime 7 days away: Checkout allowed and proceeded normally. Showtime started 20 minutes ago: Checkout blocked with message indicating ticket sales close 10 minutes after start. </t>
+  </si>
+  <si>
+    <t>QA Tester (Functional Validation)</t>
   </si>
   <si>
     <t>PreventDoubleSellingIntegration_1</t>
@@ -164,6 +147,12 @@
     <t>Seat A1 is reserved/held for User 1 and is not purchasable by User 2. After User 1 purchase, A1 is marked Sold. User 2 receives an availability error and must choose a different seat.</t>
   </si>
   <si>
+    <t>Seat A1 was held for User 1 and was not purchasable by User 2 during the hold. After User 1 purchase, A1 became Sold in inventory. User 2 received an availability error and was required to select another seat.</t>
+  </si>
+  <si>
+    <t>CI/CD Pipeline (Integration Test)</t>
+  </si>
+  <si>
     <t>BotPreventionSecurity_1</t>
   </si>
   <si>
@@ -187,7 +176,19 @@
     <t>System rate-limits excessive requests and/or prompts a human verification challenge. If verification is failed, checkout remains blocked. After passing verification (or waiting out rate limit), legitimate checkout can proceed. Security event is logged for admin review.</t>
   </si>
   <si>
+    <t>High-rate request behavior activated rate limiting and a human verification challenge. Checkout remained blocked until the challenge was passed / rate limit expired. A security event was recorded in the admin logs.</t>
+  </si>
+  <si>
+    <t>Security Tester / Pentester</t>
+  </si>
+  <si>
     <t>AdminAccessDenial_1</t>
+  </si>
+  <si>
+    <t>Admin_Module</t>
+  </si>
+  <si>
+    <t>P0</t>
   </si>
   <si>
     <t>Verify that a non-admin user cannot access the admin panel and that the event is correctly logged.</t>
@@ -208,13 +209,14 @@
     <t>Access denied message</t>
   </si>
   <si>
-    <t>Pentester</t>
+    <t>Security Test /
+Pentester</t>
   </si>
   <si>
     <t>PaymentFailure_1</t>
   </si>
   <si>
-    <t>Order_Payment_Module</t>
+    <t>Checkout_Module</t>
   </si>
   <si>
     <t>Verify that a failed payment does not finalize the order, releases the seat hold, and logs the failure event.</t>
@@ -237,13 +239,89 @@
     <t>Seat is available, and no confirmation number</t>
   </si>
   <si>
-    <t>DiscountPricing_1</t>
-  </si>
-  <si>
     <t xml:space="preserve">User </t>
   </si>
   <si>
+    <t>DiscountTicketPricing_1</t>
+  </si>
+  <si>
+    <t>Pricing_Module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify that each discount ticket type applies the correct price reduction and the final total correctly reflects the discount accurately before checkout.
+</t>
+  </si>
+  <si>
+    <t>Ticket pricing and discounts loaded, atleast one valid showtime active within the purchasing window and the user is on the seat selection/checkout page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Select a showtime and go to seat selection.
+2. Select Adult ticket type 
+3. Select Child ticket type 
+4. Select Senior ticket type 
+5. Select Student ticket type 
+6. In checkout verify that it shows the total original price, the discount and the new updated price for each ticket type.
+</t>
+  </si>
+  <si>
+    <t>Each ticket type displays a distinct price that macthes the disccounts. The totla updated correctly for each selection, the old pirce is striked out and greyed, the new price is in bold.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Verdana"/>
+        <color rgb="FF333333"/>
+        <sz val="9.0"/>
+      </rPr>
+      <t xml:space="preserve">Discounts correctly applied and </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Verdana"/>
+        <b/>
+        <color rgb="FF333333"/>
+        <sz val="9.0"/>
+      </rPr>
+      <t xml:space="preserve">easily </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Verdana"/>
+        <color rgb="FF333333"/>
+        <sz val="9.0"/>
+      </rPr>
+      <t xml:space="preserve">visible </t>
+    </r>
+  </si>
+  <si>
+    <t>CI/CD Pipeline 
+(Unit Test)</t>
+  </si>
+  <si>
     <t>SeatHoldTimer_1</t>
+  </si>
+  <si>
+    <t>Verify that a temporarily held seat is automatically released back to available in the seat inventory after the adjustable hold timer expires without a completed payment.</t>
+  </si>
+  <si>
+    <t>Valid showtime exists with at leas tone available seat, user is on seat slection page and the hold timer is configured to 5 minutes.</t>
+  </si>
+  <si>
+    <t>1. Select a available seat and go to checkout
+2. Confirm the seat shows held on the seat map
+3. Allow the 5 minute hold timer to expire without completing the payment
+4. Refresh the seat map
+5. Verify the seat status</t>
+  </si>
+  <si>
+    <t>After the hold timer expires the seat returns its status back to available on the seat map and can be selcted by users again. No order created or payment going through.</t>
+  </si>
+  <si>
+    <t>Seat returned to available after the hold expired</t>
+  </si>
+  <si>
+    <t>CI/CD Pipeline 
+(Integration Test)</t>
   </si>
   <si>
     <t>RefundRequest_1</t>
@@ -275,9 +353,6 @@
   </si>
   <si>
     <t>GuestCheckout_1</t>
-  </si>
-  <si>
-    <t>Checkout_Module</t>
   </si>
   <si>
     <t>Verify that a Guest User is able to complete a ticket purchase without needing an account</t>
@@ -303,9 +378,6 @@
   <si>
     <t>DiscountCode
 Validation_1</t>
-  </si>
-  <si>
-    <t>Pricing_Module</t>
   </si>
   <si>
     <t xml:space="preserve">Verify if a discount code is expired or invalid, showing appropriate errors for each one. </t>
@@ -457,7 +529,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -467,14 +539,6 @@
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -484,8 +548,19 @@
     <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -505,7 +580,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Victor Lopez" id="{fb3c67f4-c2b9-4e5f-8dae-10585fa6b1c3}" providerId="google-sheets"/>
+  <x18tc:person displayName="Victor Lopez" id="{8e395d96-0f77-4a6a-b11e-09ddefdf5e6e}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -705,7 +780,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A3" dT="2026-03-18T03:00:40.00" personId="{fb3c67f4-c2b9-4e5f-8dae-10585fa6b1c3}" id="{dac5ceab-4fcd-43b1-aa9a-912570d825cc}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-03-18T03:00:40.00" personId="{8e395d96-0f77-4a6a-b11e-09ddefdf5e6e}" id="{163cf64a-9a5e-4384-8ab6-10911567c6be}" done="0">
     <x18tc:text xml:space="preserve">Pascal case, underscores for spaces.
 P0 for security testing or anything that is website breaking
 P1 for functionality 
@@ -810,396 +885,427 @@
       <c r="I3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" ht="90.0" customHeight="1">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="E4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="F4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="G4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="H4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="I4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="5"/>
     </row>
     <row r="5" ht="90.0" customHeight="1">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>22</v>
+      <c r="B5" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="E5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="F5" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="5"/>
+      <c r="G5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="6" ht="90.0" customHeight="1">
-      <c r="A6" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="10" t="s">
+      <c r="A6" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="B6" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="6"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="5"/>
+      <c r="D6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="7" ht="90.0" customHeight="1">
-      <c r="A7" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="G7" s="10" t="s">
+      <c r="A7" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="H7" s="6"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="5"/>
+      <c r="B7" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="8" ht="90.0" customHeight="1">
-      <c r="A8" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="9" t="s">
+      <c r="A8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="I8" s="8"/>
-      <c r="J8" s="9" t="s">
-        <v>52</v>
+      <c r="D8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="9" ht="90.0" customHeight="1">
-      <c r="A9" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="I9" s="8"/>
-      <c r="J9" s="5"/>
+      <c r="A9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="10" ht="90.0" customHeight="1">
-      <c r="A10" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="9" t="s">
-        <v>61</v>
+      <c r="A10" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="11" ht="90.0" customHeight="1">
-      <c r="A11" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="5"/>
+      <c r="A11" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="I11" s="10"/>
+      <c r="J11" s="5" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="12" ht="90.0" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="I12" s="8"/>
-      <c r="J12" s="9" t="s">
-        <v>70</v>
+      <c r="A12" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="I12" s="10"/>
+      <c r="J12" s="5" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="13" ht="90.0" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="I13" s="8"/>
-      <c r="J13" s="9" t="s">
-        <v>70</v>
+      <c r="A13" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="I13" s="10"/>
+      <c r="J13" s="5" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="14" ht="90.0" customHeight="1">
-      <c r="A14" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="H14" s="10" t="s">
+      <c r="A14" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="I14" s="10"/>
+      <c r="J14" s="5" t="s">
         <v>84</v>
-      </c>
-      <c r="I14" s="8"/>
-      <c r="J14" s="9" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="15" ht="90.0" customHeight="1">
-      <c r="A15" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="I15" s="8"/>
-      <c r="J15" s="9" t="s">
-        <v>70</v>
-      </c>
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="11"/>
     </row>
     <row r="16" ht="90.0" customHeight="1">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="5"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="11"/>
     </row>
     <row r="17" ht="90.0" customHeight="1">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="5"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="11"/>
     </row>
     <row r="18" ht="90.0" customHeight="1">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="5"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="11"/>
     </row>
     <row r="19" ht="90.0" customHeight="1">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="5"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="11"/>
     </row>
     <row r="20" ht="90.0" customHeight="1">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="5"/>
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="11"/>
     </row>
-    <row r="21" ht="90.0" customHeight="1">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="5"/>
-    </row>
+    <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1"/>
@@ -2178,7 +2284,6 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>